<commit_message>
fix(productos): postprocess-transversal — el contador existente se reconoce por fórmula (no solo por etiqueta) y nunca se escribe un segundo; etiqueta original conservada; reparación exacta del Progreso (%) del onboarding (filas literales → celdas)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016924EP7QJuq6BNFj8S7Fks
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-gestion-personal/01-cuadrante-turnos-semanal.xlsx
+++ b/astro-site/public/dl/kit-gestion-personal/01-cuadrante-turnos-semanal.xlsx
@@ -1,19 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadrante Semanal" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadrante Mensual" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Cuadrante Semanal" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Cuadrante Mensual" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Cuadrante Semanal'!$5:$5</definedName>
-  </definedNames>
+  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -170,57 +168,57 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
   </cellStyleXfs>
   <cellXfs count="21">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="5" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="6" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="7" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="1" fillId="8" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="1" fillId="8" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="1" fillId="8" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -580,16 +578,15 @@
   <sheetPr>
     <tabColor rgb="00FFD700"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="B2:B20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="80" customWidth="1" min="2" max="2"/>
+    <col customWidth="1" max="1" min="1" width="3"/>
+    <col customWidth="1" max="2" min="2" width="80"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -597,7 +594,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -633,7 +629,9 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
+    <row r="9">
+      <c r="B9" t="inlineStr"/>
+    </row>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -662,7 +660,9 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
+    <row r="14">
+      <c r="B14" t="inlineStr"/>
+    </row>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -705,25 +705,8 @@
         </is>
       </c>
     </row>
-    <row r="21"/>
-    <row r="22">
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-gestion-personal · info@aichef.pro</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -732,21 +715,21 @@
   <sheetPr>
     <tabColor rgb="001565C0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col customWidth="1" max="1" min="1" width="22"/>
+    <col customWidth="1" max="2" min="2" width="14"/>
+    <col customWidth="1" max="3" min="3" width="14"/>
+    <col customWidth="1" max="4" min="4" width="14"/>
+    <col customWidth="1" max="5" min="5" width="14"/>
+    <col customWidth="1" max="6" min="6" width="14"/>
+    <col customWidth="1" max="7" min="7" width="14"/>
+    <col customWidth="1" max="8" min="8" width="14"/>
+    <col customWidth="1" max="9" min="9" width="14"/>
+    <col customWidth="1" max="10" min="10" width="16"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -790,7 +773,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
@@ -854,7 +836,7 @@
       <c r="H6" s="13" t="n"/>
       <c r="I6" s="14">
         <f>IF(B6="M",8,IF(B6="T",8,IF(B6="N",8,IF(B6="P",9,0))))+IF(C6="M",8,IF(C6="T",8,IF(C6="N",8,IF(C6="P",9,0))))+IF(D6="M",8,IF(D6="T",8,IF(D6="N",8,IF(D6="P",9,0))))+IF(E6="M",8,IF(E6="T",8,IF(E6="N",8,IF(E6="P",9,0))))+IF(F6="M",8,IF(F6="T",8,IF(F6="N",8,IF(F6="P",9,0))))+IF(G6="M",8,IF(G6="T",8,IF(G6="N",8,IF(G6="P",9,0))))+IF(H6="M",8,IF(H6="T",8,IF(H6="N",8,IF(H6="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J6" s="15">
         <f>IF(I6&gt;40,"⚠ EXCESO",IF(I6&gt;0,"OK",""))</f>
@@ -872,7 +854,7 @@
       <c r="H7" s="13" t="n"/>
       <c r="I7" s="14">
         <f>IF(B7="M",8,IF(B7="T",8,IF(B7="N",8,IF(B7="P",9,0))))+IF(C7="M",8,IF(C7="T",8,IF(C7="N",8,IF(C7="P",9,0))))+IF(D7="M",8,IF(D7="T",8,IF(D7="N",8,IF(D7="P",9,0))))+IF(E7="M",8,IF(E7="T",8,IF(E7="N",8,IF(E7="P",9,0))))+IF(F7="M",8,IF(F7="T",8,IF(F7="N",8,IF(F7="P",9,0))))+IF(G7="M",8,IF(G7="T",8,IF(G7="N",8,IF(G7="P",9,0))))+IF(H7="M",8,IF(H7="T",8,IF(H7="N",8,IF(H7="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J7" s="15">
         <f>IF(I7&gt;40,"⚠ EXCESO",IF(I7&gt;0,"OK",""))</f>
@@ -890,7 +872,7 @@
       <c r="H8" s="13" t="n"/>
       <c r="I8" s="14">
         <f>IF(B8="M",8,IF(B8="T",8,IF(B8="N",8,IF(B8="P",9,0))))+IF(C8="M",8,IF(C8="T",8,IF(C8="N",8,IF(C8="P",9,0))))+IF(D8="M",8,IF(D8="T",8,IF(D8="N",8,IF(D8="P",9,0))))+IF(E8="M",8,IF(E8="T",8,IF(E8="N",8,IF(E8="P",9,0))))+IF(F8="M",8,IF(F8="T",8,IF(F8="N",8,IF(F8="P",9,0))))+IF(G8="M",8,IF(G8="T",8,IF(G8="N",8,IF(G8="P",9,0))))+IF(H8="M",8,IF(H8="T",8,IF(H8="N",8,IF(H8="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J8" s="15">
         <f>IF(I8&gt;40,"⚠ EXCESO",IF(I8&gt;0,"OK",""))</f>
@@ -908,7 +890,7 @@
       <c r="H9" s="13" t="n"/>
       <c r="I9" s="14">
         <f>IF(B9="M",8,IF(B9="T",8,IF(B9="N",8,IF(B9="P",9,0))))+IF(C9="M",8,IF(C9="T",8,IF(C9="N",8,IF(C9="P",9,0))))+IF(D9="M",8,IF(D9="T",8,IF(D9="N",8,IF(D9="P",9,0))))+IF(E9="M",8,IF(E9="T",8,IF(E9="N",8,IF(E9="P",9,0))))+IF(F9="M",8,IF(F9="T",8,IF(F9="N",8,IF(F9="P",9,0))))+IF(G9="M",8,IF(G9="T",8,IF(G9="N",8,IF(G9="P",9,0))))+IF(H9="M",8,IF(H9="T",8,IF(H9="N",8,IF(H9="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J9" s="15">
         <f>IF(I9&gt;40,"⚠ EXCESO",IF(I9&gt;0,"OK",""))</f>
@@ -926,7 +908,7 @@
       <c r="H10" s="13" t="n"/>
       <c r="I10" s="14">
         <f>IF(B10="M",8,IF(B10="T",8,IF(B10="N",8,IF(B10="P",9,0))))+IF(C10="M",8,IF(C10="T",8,IF(C10="N",8,IF(C10="P",9,0))))+IF(D10="M",8,IF(D10="T",8,IF(D10="N",8,IF(D10="P",9,0))))+IF(E10="M",8,IF(E10="T",8,IF(E10="N",8,IF(E10="P",9,0))))+IF(F10="M",8,IF(F10="T",8,IF(F10="N",8,IF(F10="P",9,0))))+IF(G10="M",8,IF(G10="T",8,IF(G10="N",8,IF(G10="P",9,0))))+IF(H10="M",8,IF(H10="T",8,IF(H10="N",8,IF(H10="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J10" s="15">
         <f>IF(I10&gt;40,"⚠ EXCESO",IF(I10&gt;0,"OK",""))</f>
@@ -944,7 +926,7 @@
       <c r="H11" s="13" t="n"/>
       <c r="I11" s="14">
         <f>IF(B11="M",8,IF(B11="T",8,IF(B11="N",8,IF(B11="P",9,0))))+IF(C11="M",8,IF(C11="T",8,IF(C11="N",8,IF(C11="P",9,0))))+IF(D11="M",8,IF(D11="T",8,IF(D11="N",8,IF(D11="P",9,0))))+IF(E11="M",8,IF(E11="T",8,IF(E11="N",8,IF(E11="P",9,0))))+IF(F11="M",8,IF(F11="T",8,IF(F11="N",8,IF(F11="P",9,0))))+IF(G11="M",8,IF(G11="T",8,IF(G11="N",8,IF(G11="P",9,0))))+IF(H11="M",8,IF(H11="T",8,IF(H11="N",8,IF(H11="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J11" s="15">
         <f>IF(I11&gt;40,"⚠ EXCESO",IF(I11&gt;0,"OK",""))</f>
@@ -962,7 +944,7 @@
       <c r="H12" s="13" t="n"/>
       <c r="I12" s="14">
         <f>IF(B12="M",8,IF(B12="T",8,IF(B12="N",8,IF(B12="P",9,0))))+IF(C12="M",8,IF(C12="T",8,IF(C12="N",8,IF(C12="P",9,0))))+IF(D12="M",8,IF(D12="T",8,IF(D12="N",8,IF(D12="P",9,0))))+IF(E12="M",8,IF(E12="T",8,IF(E12="N",8,IF(E12="P",9,0))))+IF(F12="M",8,IF(F12="T",8,IF(F12="N",8,IF(F12="P",9,0))))+IF(G12="M",8,IF(G12="T",8,IF(G12="N",8,IF(G12="P",9,0))))+IF(H12="M",8,IF(H12="T",8,IF(H12="N",8,IF(H12="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J12" s="15">
         <f>IF(I12&gt;40,"⚠ EXCESO",IF(I12&gt;0,"OK",""))</f>
@@ -980,7 +962,7 @@
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="14">
         <f>IF(B13="M",8,IF(B13="T",8,IF(B13="N",8,IF(B13="P",9,0))))+IF(C13="M",8,IF(C13="T",8,IF(C13="N",8,IF(C13="P",9,0))))+IF(D13="M",8,IF(D13="T",8,IF(D13="N",8,IF(D13="P",9,0))))+IF(E13="M",8,IF(E13="T",8,IF(E13="N",8,IF(E13="P",9,0))))+IF(F13="M",8,IF(F13="T",8,IF(F13="N",8,IF(F13="P",9,0))))+IF(G13="M",8,IF(G13="T",8,IF(G13="N",8,IF(G13="P",9,0))))+IF(H13="M",8,IF(H13="T",8,IF(H13="N",8,IF(H13="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J13" s="15">
         <f>IF(I13&gt;40,"⚠ EXCESO",IF(I13&gt;0,"OK",""))</f>
@@ -998,7 +980,7 @@
       <c r="H14" s="13" t="n"/>
       <c r="I14" s="14">
         <f>IF(B14="M",8,IF(B14="T",8,IF(B14="N",8,IF(B14="P",9,0))))+IF(C14="M",8,IF(C14="T",8,IF(C14="N",8,IF(C14="P",9,0))))+IF(D14="M",8,IF(D14="T",8,IF(D14="N",8,IF(D14="P",9,0))))+IF(E14="M",8,IF(E14="T",8,IF(E14="N",8,IF(E14="P",9,0))))+IF(F14="M",8,IF(F14="T",8,IF(F14="N",8,IF(F14="P",9,0))))+IF(G14="M",8,IF(G14="T",8,IF(G14="N",8,IF(G14="P",9,0))))+IF(H14="M",8,IF(H14="T",8,IF(H14="N",8,IF(H14="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J14" s="15">
         <f>IF(I14&gt;40,"⚠ EXCESO",IF(I14&gt;0,"OK",""))</f>
@@ -1016,7 +998,7 @@
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="14">
         <f>IF(B15="M",8,IF(B15="T",8,IF(B15="N",8,IF(B15="P",9,0))))+IF(C15="M",8,IF(C15="T",8,IF(C15="N",8,IF(C15="P",9,0))))+IF(D15="M",8,IF(D15="T",8,IF(D15="N",8,IF(D15="P",9,0))))+IF(E15="M",8,IF(E15="T",8,IF(E15="N",8,IF(E15="P",9,0))))+IF(F15="M",8,IF(F15="T",8,IF(F15="N",8,IF(F15="P",9,0))))+IF(G15="M",8,IF(G15="T",8,IF(G15="N",8,IF(G15="P",9,0))))+IF(H15="M",8,IF(H15="T",8,IF(H15="N",8,IF(H15="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J15" s="15">
         <f>IF(I15&gt;40,"⚠ EXCESO",IF(I15&gt;0,"OK",""))</f>
@@ -1034,7 +1016,7 @@
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="14">
         <f>IF(B16="M",8,IF(B16="T",8,IF(B16="N",8,IF(B16="P",9,0))))+IF(C16="M",8,IF(C16="T",8,IF(C16="N",8,IF(C16="P",9,0))))+IF(D16="M",8,IF(D16="T",8,IF(D16="N",8,IF(D16="P",9,0))))+IF(E16="M",8,IF(E16="T",8,IF(E16="N",8,IF(E16="P",9,0))))+IF(F16="M",8,IF(F16="T",8,IF(F16="N",8,IF(F16="P",9,0))))+IF(G16="M",8,IF(G16="T",8,IF(G16="N",8,IF(G16="P",9,0))))+IF(H16="M",8,IF(H16="T",8,IF(H16="N",8,IF(H16="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J16" s="15">
         <f>IF(I16&gt;40,"⚠ EXCESO",IF(I16&gt;0,"OK",""))</f>
@@ -1052,7 +1034,7 @@
       <c r="H17" s="13" t="n"/>
       <c r="I17" s="14">
         <f>IF(B17="M",8,IF(B17="T",8,IF(B17="N",8,IF(B17="P",9,0))))+IF(C17="M",8,IF(C17="T",8,IF(C17="N",8,IF(C17="P",9,0))))+IF(D17="M",8,IF(D17="T",8,IF(D17="N",8,IF(D17="P",9,0))))+IF(E17="M",8,IF(E17="T",8,IF(E17="N",8,IF(E17="P",9,0))))+IF(F17="M",8,IF(F17="T",8,IF(F17="N",8,IF(F17="P",9,0))))+IF(G17="M",8,IF(G17="T",8,IF(G17="N",8,IF(G17="P",9,0))))+IF(H17="M",8,IF(H17="T",8,IF(H17="N",8,IF(H17="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J17" s="15">
         <f>IF(I17&gt;40,"⚠ EXCESO",IF(I17&gt;0,"OK",""))</f>
@@ -1070,7 +1052,7 @@
       <c r="H18" s="13" t="n"/>
       <c r="I18" s="14">
         <f>IF(B18="M",8,IF(B18="T",8,IF(B18="N",8,IF(B18="P",9,0))))+IF(C18="M",8,IF(C18="T",8,IF(C18="N",8,IF(C18="P",9,0))))+IF(D18="M",8,IF(D18="T",8,IF(D18="N",8,IF(D18="P",9,0))))+IF(E18="M",8,IF(E18="T",8,IF(E18="N",8,IF(E18="P",9,0))))+IF(F18="M",8,IF(F18="T",8,IF(F18="N",8,IF(F18="P",9,0))))+IF(G18="M",8,IF(G18="T",8,IF(G18="N",8,IF(G18="P",9,0))))+IF(H18="M",8,IF(H18="T",8,IF(H18="N",8,IF(H18="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J18" s="15">
         <f>IF(I18&gt;40,"⚠ EXCESO",IF(I18&gt;0,"OK",""))</f>
@@ -1088,7 +1070,7 @@
       <c r="H19" s="13" t="n"/>
       <c r="I19" s="14">
         <f>IF(B19="M",8,IF(B19="T",8,IF(B19="N",8,IF(B19="P",9,0))))+IF(C19="M",8,IF(C19="T",8,IF(C19="N",8,IF(C19="P",9,0))))+IF(D19="M",8,IF(D19="T",8,IF(D19="N",8,IF(D19="P",9,0))))+IF(E19="M",8,IF(E19="T",8,IF(E19="N",8,IF(E19="P",9,0))))+IF(F19="M",8,IF(F19="T",8,IF(F19="N",8,IF(F19="P",9,0))))+IF(G19="M",8,IF(G19="T",8,IF(G19="N",8,IF(G19="P",9,0))))+IF(H19="M",8,IF(H19="T",8,IF(H19="N",8,IF(H19="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J19" s="15">
         <f>IF(I19&gt;40,"⚠ EXCESO",IF(I19&gt;0,"OK",""))</f>
@@ -1106,7 +1088,7 @@
       <c r="H20" s="13" t="n"/>
       <c r="I20" s="14">
         <f>IF(B20="M",8,IF(B20="T",8,IF(B20="N",8,IF(B20="P",9,0))))+IF(C20="M",8,IF(C20="T",8,IF(C20="N",8,IF(C20="P",9,0))))+IF(D20="M",8,IF(D20="T",8,IF(D20="N",8,IF(D20="P",9,0))))+IF(E20="M",8,IF(E20="T",8,IF(E20="N",8,IF(E20="P",9,0))))+IF(F20="M",8,IF(F20="T",8,IF(F20="N",8,IF(F20="P",9,0))))+IF(G20="M",8,IF(G20="T",8,IF(G20="N",8,IF(G20="P",9,0))))+IF(H20="M",8,IF(H20="T",8,IF(H20="N",8,IF(H20="P",9,0))))</f>
-        <v>0.0</v>
+        <v/>
       </c>
       <c r="J20" s="15">
         <f>IF(I20&gt;40,"⚠ EXCESO",IF(I20&gt;0,"OK",""))</f>
@@ -1121,10 +1103,9 @@
       </c>
       <c r="I21" s="14">
         <f>SUM(I6:I20)</f>
-        <v>0.0</v>
-      </c>
-    </row>
-    <row r="22"/>
+        <v/>
+      </c>
+    </row>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
@@ -1139,20 +1120,11 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa M, T, N, P o L" prompt="M=Mañana, T=Tarde, N=Noche, P=Partido, L=Libre" type="list">
+    <dataValidation allowBlank="1" error="Usa M, T, N, P o L" prompt="M=Mañana, T=Tarde, N=Noche, P=Partido, L=Libre" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20" type="list">
       <formula1>"M,T,N,P,L"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
 
@@ -1161,20 +1133,20 @@
   <sheetPr>
     <tabColor rgb="000D47A1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr fitToPage="1"/>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col customWidth="1" max="1" min="1" width="22"/>
+    <col customWidth="1" max="2" min="2" width="12"/>
+    <col customWidth="1" max="3" min="3" width="12"/>
+    <col customWidth="1" max="4" min="4" width="12"/>
+    <col customWidth="1" max="5" min="5" width="12"/>
+    <col customWidth="1" max="6" min="6" width="12"/>
+    <col customWidth="1" max="7" min="7" width="12"/>
+    <col customWidth="1" max="8" min="8" width="12"/>
+    <col customWidth="1" max="9" min="9" width="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1410,8 +1382,6 @@
       <c r="H19" s="20" t="n"/>
       <c r="I19" s="20" t="n"/>
     </row>
-    <row r="20"/>
-    <row r="21"/>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
         <is>
@@ -1631,8 +1601,6 @@
       <c r="H38" s="20" t="n"/>
       <c r="I38" s="20" t="n"/>
     </row>
-    <row r="39"/>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
@@ -1852,8 +1820,6 @@
       <c r="H57" s="20" t="n"/>
       <c r="I57" s="20" t="n"/>
     </row>
-    <row r="58"/>
-    <row r="59"/>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
@@ -2073,9 +2039,6 @@
       <c r="H76" s="20" t="n"/>
       <c r="I76" s="20" t="n"/>
     </row>
-    <row r="77"/>
-    <row r="78"/>
-    <row r="79"/>
     <row r="80">
       <c r="A80" s="17" t="inlineStr">
         <is>
@@ -2089,15 +2052,6 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A80:I80"/>
   </mergeCells>
-  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
-  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
-  <headerFooter>
-    <oddHeader/>
-    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(productos): kit-gestion-personal re-saneado — onboarding con un solo contador (etiqueta original) y Progreso (%) real
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016924EP7QJuq6BNFj8S7Fks
</commit_message>
<xml_diff>
--- a/astro-site/public/dl/kit-gestion-personal/01-cuadrante-turnos-semanal.xlsx
+++ b/astro-site/public/dl/kit-gestion-personal/01-cuadrante-turnos-semanal.xlsx
@@ -1,17 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Cuadrante Semanal" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cuadrante Mensual" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadrante Semanal" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Cuadrante Mensual" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'Cuadrante Semanal'!$5:$5</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -168,57 +170,57 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="21">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="0" fillId="2" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="3" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="5" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="0" fillId="6" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="7" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="8" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="1" fillId="8" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf applyAlignment="1" borderId="1" fillId="8" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf applyAlignment="1" borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle builtinId="0" hidden="0" name="Normal" xfId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium9"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -578,15 +580,16 @@
   <sheetPr>
     <tabColor rgb="00FFD700"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:B20"/>
+  <dimension ref="A1:B22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="3"/>
-    <col customWidth="1" max="2" min="2" width="80"/>
+    <col width="3" customWidth="1" min="1" max="1"/>
+    <col width="80" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -594,6 +597,7 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="B4" s="2" t="inlineStr">
         <is>
@@ -629,9 +633,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="B9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="2" t="inlineStr">
         <is>
@@ -660,9 +662,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="B15" s="2" t="inlineStr">
         <is>
@@ -705,8 +705,25 @@
         </is>
       </c>
     </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Versión 1.1 · agosto 2026 · aichef.pro/kit-gestion-personal · info@aichef.pro</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -715,21 +732,21 @@
   <sheetPr>
     <tabColor rgb="001565C0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:J23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="22"/>
-    <col customWidth="1" max="2" min="2" width="14"/>
-    <col customWidth="1" max="3" min="3" width="14"/>
-    <col customWidth="1" max="4" min="4" width="14"/>
-    <col customWidth="1" max="5" min="5" width="14"/>
-    <col customWidth="1" max="6" min="6" width="14"/>
-    <col customWidth="1" max="7" min="7" width="14"/>
-    <col customWidth="1" max="8" min="8" width="14"/>
-    <col customWidth="1" max="9" min="9" width="14"/>
-    <col customWidth="1" max="10" min="10" width="16"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -773,6 +790,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="11" t="inlineStr">
         <is>
@@ -836,7 +854,7 @@
       <c r="H6" s="13" t="n"/>
       <c r="I6" s="14">
         <f>IF(B6="M",8,IF(B6="T",8,IF(B6="N",8,IF(B6="P",9,0))))+IF(C6="M",8,IF(C6="T",8,IF(C6="N",8,IF(C6="P",9,0))))+IF(D6="M",8,IF(D6="T",8,IF(D6="N",8,IF(D6="P",9,0))))+IF(E6="M",8,IF(E6="T",8,IF(E6="N",8,IF(E6="P",9,0))))+IF(F6="M",8,IF(F6="T",8,IF(F6="N",8,IF(F6="P",9,0))))+IF(G6="M",8,IF(G6="T",8,IF(G6="N",8,IF(G6="P",9,0))))+IF(H6="M",8,IF(H6="T",8,IF(H6="N",8,IF(H6="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J6" s="15">
         <f>IF(I6&gt;40,"⚠ EXCESO",IF(I6&gt;0,"OK",""))</f>
@@ -854,7 +872,7 @@
       <c r="H7" s="13" t="n"/>
       <c r="I7" s="14">
         <f>IF(B7="M",8,IF(B7="T",8,IF(B7="N",8,IF(B7="P",9,0))))+IF(C7="M",8,IF(C7="T",8,IF(C7="N",8,IF(C7="P",9,0))))+IF(D7="M",8,IF(D7="T",8,IF(D7="N",8,IF(D7="P",9,0))))+IF(E7="M",8,IF(E7="T",8,IF(E7="N",8,IF(E7="P",9,0))))+IF(F7="M",8,IF(F7="T",8,IF(F7="N",8,IF(F7="P",9,0))))+IF(G7="M",8,IF(G7="T",8,IF(G7="N",8,IF(G7="P",9,0))))+IF(H7="M",8,IF(H7="T",8,IF(H7="N",8,IF(H7="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J7" s="15">
         <f>IF(I7&gt;40,"⚠ EXCESO",IF(I7&gt;0,"OK",""))</f>
@@ -872,7 +890,7 @@
       <c r="H8" s="13" t="n"/>
       <c r="I8" s="14">
         <f>IF(B8="M",8,IF(B8="T",8,IF(B8="N",8,IF(B8="P",9,0))))+IF(C8="M",8,IF(C8="T",8,IF(C8="N",8,IF(C8="P",9,0))))+IF(D8="M",8,IF(D8="T",8,IF(D8="N",8,IF(D8="P",9,0))))+IF(E8="M",8,IF(E8="T",8,IF(E8="N",8,IF(E8="P",9,0))))+IF(F8="M",8,IF(F8="T",8,IF(F8="N",8,IF(F8="P",9,0))))+IF(G8="M",8,IF(G8="T",8,IF(G8="N",8,IF(G8="P",9,0))))+IF(H8="M",8,IF(H8="T",8,IF(H8="N",8,IF(H8="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J8" s="15">
         <f>IF(I8&gt;40,"⚠ EXCESO",IF(I8&gt;0,"OK",""))</f>
@@ -890,7 +908,7 @@
       <c r="H9" s="13" t="n"/>
       <c r="I9" s="14">
         <f>IF(B9="M",8,IF(B9="T",8,IF(B9="N",8,IF(B9="P",9,0))))+IF(C9="M",8,IF(C9="T",8,IF(C9="N",8,IF(C9="P",9,0))))+IF(D9="M",8,IF(D9="T",8,IF(D9="N",8,IF(D9="P",9,0))))+IF(E9="M",8,IF(E9="T",8,IF(E9="N",8,IF(E9="P",9,0))))+IF(F9="M",8,IF(F9="T",8,IF(F9="N",8,IF(F9="P",9,0))))+IF(G9="M",8,IF(G9="T",8,IF(G9="N",8,IF(G9="P",9,0))))+IF(H9="M",8,IF(H9="T",8,IF(H9="N",8,IF(H9="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J9" s="15">
         <f>IF(I9&gt;40,"⚠ EXCESO",IF(I9&gt;0,"OK",""))</f>
@@ -908,7 +926,7 @@
       <c r="H10" s="13" t="n"/>
       <c r="I10" s="14">
         <f>IF(B10="M",8,IF(B10="T",8,IF(B10="N",8,IF(B10="P",9,0))))+IF(C10="M",8,IF(C10="T",8,IF(C10="N",8,IF(C10="P",9,0))))+IF(D10="M",8,IF(D10="T",8,IF(D10="N",8,IF(D10="P",9,0))))+IF(E10="M",8,IF(E10="T",8,IF(E10="N",8,IF(E10="P",9,0))))+IF(F10="M",8,IF(F10="T",8,IF(F10="N",8,IF(F10="P",9,0))))+IF(G10="M",8,IF(G10="T",8,IF(G10="N",8,IF(G10="P",9,0))))+IF(H10="M",8,IF(H10="T",8,IF(H10="N",8,IF(H10="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J10" s="15">
         <f>IF(I10&gt;40,"⚠ EXCESO",IF(I10&gt;0,"OK",""))</f>
@@ -926,7 +944,7 @@
       <c r="H11" s="13" t="n"/>
       <c r="I11" s="14">
         <f>IF(B11="M",8,IF(B11="T",8,IF(B11="N",8,IF(B11="P",9,0))))+IF(C11="M",8,IF(C11="T",8,IF(C11="N",8,IF(C11="P",9,0))))+IF(D11="M",8,IF(D11="T",8,IF(D11="N",8,IF(D11="P",9,0))))+IF(E11="M",8,IF(E11="T",8,IF(E11="N",8,IF(E11="P",9,0))))+IF(F11="M",8,IF(F11="T",8,IF(F11="N",8,IF(F11="P",9,0))))+IF(G11="M",8,IF(G11="T",8,IF(G11="N",8,IF(G11="P",9,0))))+IF(H11="M",8,IF(H11="T",8,IF(H11="N",8,IF(H11="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J11" s="15">
         <f>IF(I11&gt;40,"⚠ EXCESO",IF(I11&gt;0,"OK",""))</f>
@@ -944,7 +962,7 @@
       <c r="H12" s="13" t="n"/>
       <c r="I12" s="14">
         <f>IF(B12="M",8,IF(B12="T",8,IF(B12="N",8,IF(B12="P",9,0))))+IF(C12="M",8,IF(C12="T",8,IF(C12="N",8,IF(C12="P",9,0))))+IF(D12="M",8,IF(D12="T",8,IF(D12="N",8,IF(D12="P",9,0))))+IF(E12="M",8,IF(E12="T",8,IF(E12="N",8,IF(E12="P",9,0))))+IF(F12="M",8,IF(F12="T",8,IF(F12="N",8,IF(F12="P",9,0))))+IF(G12="M",8,IF(G12="T",8,IF(G12="N",8,IF(G12="P",9,0))))+IF(H12="M",8,IF(H12="T",8,IF(H12="N",8,IF(H12="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J12" s="15">
         <f>IF(I12&gt;40,"⚠ EXCESO",IF(I12&gt;0,"OK",""))</f>
@@ -962,7 +980,7 @@
       <c r="H13" s="13" t="n"/>
       <c r="I13" s="14">
         <f>IF(B13="M",8,IF(B13="T",8,IF(B13="N",8,IF(B13="P",9,0))))+IF(C13="M",8,IF(C13="T",8,IF(C13="N",8,IF(C13="P",9,0))))+IF(D13="M",8,IF(D13="T",8,IF(D13="N",8,IF(D13="P",9,0))))+IF(E13="M",8,IF(E13="T",8,IF(E13="N",8,IF(E13="P",9,0))))+IF(F13="M",8,IF(F13="T",8,IF(F13="N",8,IF(F13="P",9,0))))+IF(G13="M",8,IF(G13="T",8,IF(G13="N",8,IF(G13="P",9,0))))+IF(H13="M",8,IF(H13="T",8,IF(H13="N",8,IF(H13="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J13" s="15">
         <f>IF(I13&gt;40,"⚠ EXCESO",IF(I13&gt;0,"OK",""))</f>
@@ -980,7 +998,7 @@
       <c r="H14" s="13" t="n"/>
       <c r="I14" s="14">
         <f>IF(B14="M",8,IF(B14="T",8,IF(B14="N",8,IF(B14="P",9,0))))+IF(C14="M",8,IF(C14="T",8,IF(C14="N",8,IF(C14="P",9,0))))+IF(D14="M",8,IF(D14="T",8,IF(D14="N",8,IF(D14="P",9,0))))+IF(E14="M",8,IF(E14="T",8,IF(E14="N",8,IF(E14="P",9,0))))+IF(F14="M",8,IF(F14="T",8,IF(F14="N",8,IF(F14="P",9,0))))+IF(G14="M",8,IF(G14="T",8,IF(G14="N",8,IF(G14="P",9,0))))+IF(H14="M",8,IF(H14="T",8,IF(H14="N",8,IF(H14="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J14" s="15">
         <f>IF(I14&gt;40,"⚠ EXCESO",IF(I14&gt;0,"OK",""))</f>
@@ -998,7 +1016,7 @@
       <c r="H15" s="13" t="n"/>
       <c r="I15" s="14">
         <f>IF(B15="M",8,IF(B15="T",8,IF(B15="N",8,IF(B15="P",9,0))))+IF(C15="M",8,IF(C15="T",8,IF(C15="N",8,IF(C15="P",9,0))))+IF(D15="M",8,IF(D15="T",8,IF(D15="N",8,IF(D15="P",9,0))))+IF(E15="M",8,IF(E15="T",8,IF(E15="N",8,IF(E15="P",9,0))))+IF(F15="M",8,IF(F15="T",8,IF(F15="N",8,IF(F15="P",9,0))))+IF(G15="M",8,IF(G15="T",8,IF(G15="N",8,IF(G15="P",9,0))))+IF(H15="M",8,IF(H15="T",8,IF(H15="N",8,IF(H15="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J15" s="15">
         <f>IF(I15&gt;40,"⚠ EXCESO",IF(I15&gt;0,"OK",""))</f>
@@ -1016,7 +1034,7 @@
       <c r="H16" s="13" t="n"/>
       <c r="I16" s="14">
         <f>IF(B16="M",8,IF(B16="T",8,IF(B16="N",8,IF(B16="P",9,0))))+IF(C16="M",8,IF(C16="T",8,IF(C16="N",8,IF(C16="P",9,0))))+IF(D16="M",8,IF(D16="T",8,IF(D16="N",8,IF(D16="P",9,0))))+IF(E16="M",8,IF(E16="T",8,IF(E16="N",8,IF(E16="P",9,0))))+IF(F16="M",8,IF(F16="T",8,IF(F16="N",8,IF(F16="P",9,0))))+IF(G16="M",8,IF(G16="T",8,IF(G16="N",8,IF(G16="P",9,0))))+IF(H16="M",8,IF(H16="T",8,IF(H16="N",8,IF(H16="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J16" s="15">
         <f>IF(I16&gt;40,"⚠ EXCESO",IF(I16&gt;0,"OK",""))</f>
@@ -1034,7 +1052,7 @@
       <c r="H17" s="13" t="n"/>
       <c r="I17" s="14">
         <f>IF(B17="M",8,IF(B17="T",8,IF(B17="N",8,IF(B17="P",9,0))))+IF(C17="M",8,IF(C17="T",8,IF(C17="N",8,IF(C17="P",9,0))))+IF(D17="M",8,IF(D17="T",8,IF(D17="N",8,IF(D17="P",9,0))))+IF(E17="M",8,IF(E17="T",8,IF(E17="N",8,IF(E17="P",9,0))))+IF(F17="M",8,IF(F17="T",8,IF(F17="N",8,IF(F17="P",9,0))))+IF(G17="M",8,IF(G17="T",8,IF(G17="N",8,IF(G17="P",9,0))))+IF(H17="M",8,IF(H17="T",8,IF(H17="N",8,IF(H17="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J17" s="15">
         <f>IF(I17&gt;40,"⚠ EXCESO",IF(I17&gt;0,"OK",""))</f>
@@ -1052,7 +1070,7 @@
       <c r="H18" s="13" t="n"/>
       <c r="I18" s="14">
         <f>IF(B18="M",8,IF(B18="T",8,IF(B18="N",8,IF(B18="P",9,0))))+IF(C18="M",8,IF(C18="T",8,IF(C18="N",8,IF(C18="P",9,0))))+IF(D18="M",8,IF(D18="T",8,IF(D18="N",8,IF(D18="P",9,0))))+IF(E18="M",8,IF(E18="T",8,IF(E18="N",8,IF(E18="P",9,0))))+IF(F18="M",8,IF(F18="T",8,IF(F18="N",8,IF(F18="P",9,0))))+IF(G18="M",8,IF(G18="T",8,IF(G18="N",8,IF(G18="P",9,0))))+IF(H18="M",8,IF(H18="T",8,IF(H18="N",8,IF(H18="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J18" s="15">
         <f>IF(I18&gt;40,"⚠ EXCESO",IF(I18&gt;0,"OK",""))</f>
@@ -1070,7 +1088,7 @@
       <c r="H19" s="13" t="n"/>
       <c r="I19" s="14">
         <f>IF(B19="M",8,IF(B19="T",8,IF(B19="N",8,IF(B19="P",9,0))))+IF(C19="M",8,IF(C19="T",8,IF(C19="N",8,IF(C19="P",9,0))))+IF(D19="M",8,IF(D19="T",8,IF(D19="N",8,IF(D19="P",9,0))))+IF(E19="M",8,IF(E19="T",8,IF(E19="N",8,IF(E19="P",9,0))))+IF(F19="M",8,IF(F19="T",8,IF(F19="N",8,IF(F19="P",9,0))))+IF(G19="M",8,IF(G19="T",8,IF(G19="N",8,IF(G19="P",9,0))))+IF(H19="M",8,IF(H19="T",8,IF(H19="N",8,IF(H19="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J19" s="15">
         <f>IF(I19&gt;40,"⚠ EXCESO",IF(I19&gt;0,"OK",""))</f>
@@ -1088,7 +1106,7 @@
       <c r="H20" s="13" t="n"/>
       <c r="I20" s="14">
         <f>IF(B20="M",8,IF(B20="T",8,IF(B20="N",8,IF(B20="P",9,0))))+IF(C20="M",8,IF(C20="T",8,IF(C20="N",8,IF(C20="P",9,0))))+IF(D20="M",8,IF(D20="T",8,IF(D20="N",8,IF(D20="P",9,0))))+IF(E20="M",8,IF(E20="T",8,IF(E20="N",8,IF(E20="P",9,0))))+IF(F20="M",8,IF(F20="T",8,IF(F20="N",8,IF(F20="P",9,0))))+IF(G20="M",8,IF(G20="T",8,IF(G20="N",8,IF(G20="P",9,0))))+IF(H20="M",8,IF(H20="T",8,IF(H20="N",8,IF(H20="P",9,0))))</f>
-        <v/>
+        <v>0.0</v>
       </c>
       <c r="J20" s="15">
         <f>IF(I20&gt;40,"⚠ EXCESO",IF(I20&gt;0,"OK",""))</f>
@@ -1103,9 +1121,10 @@
       </c>
       <c r="I21" s="14">
         <f>SUM(I6:I20)</f>
-        <v/>
-      </c>
-    </row>
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="17" t="inlineStr">
         <is>
@@ -1120,11 +1139,20 @@
     <mergeCell ref="A1:J1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation allowBlank="1" error="Usa M, T, N, P o L" prompt="M=Mañana, T=Tarde, N=Noche, P=Partido, L=Libre" showDropDown="0" showErrorMessage="0" showInputMessage="0" sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20" type="list">
+    <dataValidation sqref="B6 B7 B8 B9 B10 B11 B12 B13 B14 B15 B16 B17 B18 B19 B20 C6 C7 C8 C9 C10 C11 C12 C13 C14 C15 C16 C17 C18 C19 C20 D6 D7 D8 D9 D10 D11 D12 D13 D14 D15 D16 D17 D18 D19 D20 E6 E7 E8 E9 E10 E11 E12 E13 E14 E15 E16 E17 E18 E19 E20 F6 F7 F8 F9 F10 F11 F12 F13 F14 F15 F16 F17 F18 F19 F20 G6 G7 G8 G9 G10 G11 G12 G13 G14 G15 G16 G17 G18 G19 G20 H6 H7 H8 H9 H10 H11 H12 H13 H14 H15 H16 H17 H18 H19 H20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" error="Usa M, T, N, P o L" prompt="M=Mañana, T=Tarde, N=Noche, P=Partido, L=Libre" type="list">
       <formula1>"M,T,N,P,L"</formula1>
     </dataValidation>
   </dataValidations>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
 
@@ -1133,20 +1161,20 @@
   <sheetPr>
     <tabColor rgb="000D47A1"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="A1:I80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col customWidth="1" max="1" min="1" width="22"/>
-    <col customWidth="1" max="2" min="2" width="12"/>
-    <col customWidth="1" max="3" min="3" width="12"/>
-    <col customWidth="1" max="4" min="4" width="12"/>
-    <col customWidth="1" max="5" min="5" width="12"/>
-    <col customWidth="1" max="6" min="6" width="12"/>
-    <col customWidth="1" max="7" min="7" width="12"/>
-    <col customWidth="1" max="8" min="8" width="12"/>
-    <col customWidth="1" max="9" min="9" width="12"/>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1382,6 +1410,8 @@
       <c r="H19" s="20" t="n"/>
       <c r="I19" s="20" t="n"/>
     </row>
+    <row r="20"/>
+    <row r="21"/>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
         <is>
@@ -1601,6 +1631,8 @@
       <c r="H38" s="20" t="n"/>
       <c r="I38" s="20" t="n"/>
     </row>
+    <row r="39"/>
+    <row r="40"/>
     <row r="41">
       <c r="A41" s="18" t="inlineStr">
         <is>
@@ -1820,6 +1852,8 @@
       <c r="H57" s="20" t="n"/>
       <c r="I57" s="20" t="n"/>
     </row>
+    <row r="58"/>
+    <row r="59"/>
     <row r="60">
       <c r="A60" s="18" t="inlineStr">
         <is>
@@ -2039,6 +2073,9 @@
       <c r="H76" s="20" t="n"/>
       <c r="I76" s="20" t="n"/>
     </row>
+    <row r="77"/>
+    <row r="78"/>
+    <row r="79"/>
     <row r="80">
       <c r="A80" s="17" t="inlineStr">
         <is>
@@ -2052,6 +2089,15 @@
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A80:I80"/>
   </mergeCells>
-  <pageMargins bottom="1" footer="0.5" header="0.5" left="0.75" right="0.75" top="1"/>
+  <pageMargins left="0.59" right="0.59" top="0.59" bottom="0.59" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;8 AI Chef Pro · aichef.pro · Página &amp;P de &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
 </worksheet>
 </file>
</xml_diff>